<commit_message>
Update default coins list to BTC, ETH, SOL, HYPE, DOGE, XRP, ADA, SOXL, MSTR and pre-crawl all 9 default coins
</commit_message>
<xml_diff>
--- a/data/all_exchanges_futures_margin.xlsx
+++ b/data/all_exchanges_futures_margin.xlsx
@@ -15,6 +15,7 @@
     <sheet name="HYPEUSDT" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="XRPUSDT" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="MSTRUSDT" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SOXLUSDT" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20188,4 +20189,2358 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G63"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>交易所</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>檔位</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>單位</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>倉位分級</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>最大槓桿</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>維持保證金率</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>維持金額(USDT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>50x</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>1.00%</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>200,000</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>40x</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>1.25%</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>500,000</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>25x</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>2.00%</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>1,625</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>1,000,000</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>20x</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>2.50%</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>4,125</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>2,000,000</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>15x</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>3.33%</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>12,425</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>5,000,000</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>10x</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>45,825</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>8,000,000</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>5x</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>295,825</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>20,000,000</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>4x</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>12.50%</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>495,825</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>50,000,000</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>3x</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>16.67%</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>1,329,825</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>100,000,000</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>2x</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>25.00%</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>5,494,825</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>200,000,000</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>1x</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>50.00%</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>30,494,825</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Bitget</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>100,000</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>2.50%</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Bitget</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>500,000</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>4.00%</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Bitget</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>2,000,000</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Bitget</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>5,000,000</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Bitget</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>10,000,000</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>12.50%</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Bitget</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>25,000,000</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>30.00%</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Bitget</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>50,000,000</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>60.00%</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>100,000</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>1.25%</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>150,000</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>1.67%</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>545</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>200,000</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>1,040</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>300,000</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>2.08%</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>1,200</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>400,000</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>2.17%</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>1,470</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>500,000</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>2.27%</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>1,870</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>600,000</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>2.38%</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>2,420</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>800,000</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>2.5%</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>3,140</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>1,000,000</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>2.63%</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>4,180</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>1,500,000</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>2.78%</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>5,680</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>2,000,000</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>2.94%</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>8,080</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>2,500,000</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>3.13%</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>11,880</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>3,000,000</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>3.33%</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>16,880</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>3,500,000</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>3.57%</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>24,080</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>4,000,000</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>3.85%</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>33,880</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>4,500,000</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>4.17%</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>46,680</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>5,000,000</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>4.55%</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>63,780</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>6,000,000</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>86,280</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>7,000,000</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>5.56%</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>119,880</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>MEXC</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>200x</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>0.4%</t>
+        </is>
+      </c>
+      <c r="G40" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>MEXC</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>1,200</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>50x</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>MEXC</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>11,500</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>20x</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>MEXC</t>
+        </is>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>53,000</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>10x</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
+        <is>
+          <t>5%</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>1,200</t>
+        </is>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="F44" s="11" t="inlineStr">
+        <is>
+          <t>2.00%</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>2,400</t>
+        </is>
+      </c>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>9.52</t>
+        </is>
+      </c>
+      <c r="F45" s="11" t="inlineStr">
+        <is>
+          <t>3.00%</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>3,600</t>
+        </is>
+      </c>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>9.09</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="inlineStr">
+        <is>
+          <t>4.00%</t>
+        </is>
+      </c>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>4,800</t>
+        </is>
+      </c>
+      <c r="E47" s="11" t="inlineStr">
+        <is>
+          <t>8.70</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="inlineStr">
+        <is>
+          <t>4.50%</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>6,000</t>
+        </is>
+      </c>
+      <c r="E48" s="11" t="inlineStr">
+        <is>
+          <t>8.33</t>
+        </is>
+      </c>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>5.00%</t>
+        </is>
+      </c>
+      <c r="G48" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B49" s="10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C49" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>7,200</t>
+        </is>
+      </c>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>8.00</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>5.50%</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>8,400</t>
+        </is>
+      </c>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>7.69</t>
+        </is>
+      </c>
+      <c r="F50" s="11" t="inlineStr">
+        <is>
+          <t>6.00%</t>
+        </is>
+      </c>
+      <c r="G50" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t>9,600</t>
+        </is>
+      </c>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>7.41</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>6.50%</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>10,800</t>
+        </is>
+      </c>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>7.14</t>
+        </is>
+      </c>
+      <c r="F52" s="11" t="inlineStr">
+        <is>
+          <t>7.00%</t>
+        </is>
+      </c>
+      <c r="G52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B53" s="10" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D53" s="11" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="E53" s="11" t="inlineStr">
+        <is>
+          <t>6.90</t>
+        </is>
+      </c>
+      <c r="F53" s="11" t="inlineStr">
+        <is>
+          <t>7.50%</t>
+        </is>
+      </c>
+      <c r="G53" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C54" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>13,200</t>
+        </is>
+      </c>
+      <c r="E54" s="11" t="inlineStr">
+        <is>
+          <t>6.67</t>
+        </is>
+      </c>
+      <c r="F54" s="11" t="inlineStr">
+        <is>
+          <t>8.00%</t>
+        </is>
+      </c>
+      <c r="G54" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C55" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>14,400</t>
+        </is>
+      </c>
+      <c r="E55" s="11" t="inlineStr">
+        <is>
+          <t>6.45</t>
+        </is>
+      </c>
+      <c r="F55" s="11" t="inlineStr">
+        <is>
+          <t>8.50%</t>
+        </is>
+      </c>
+      <c r="G55" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>15,600</t>
+        </is>
+      </c>
+      <c r="E56" s="11" t="inlineStr">
+        <is>
+          <t>6.25</t>
+        </is>
+      </c>
+      <c r="F56" s="11" t="inlineStr">
+        <is>
+          <t>9.00%</t>
+        </is>
+      </c>
+      <c r="G56" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B57" s="10" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr">
+        <is>
+          <t>16,800</t>
+        </is>
+      </c>
+      <c r="E57" s="11" t="inlineStr">
+        <is>
+          <t>6.06</t>
+        </is>
+      </c>
+      <c r="F57" s="11" t="inlineStr">
+        <is>
+          <t>9.50%</t>
+        </is>
+      </c>
+      <c r="G57" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C58" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>18,000</t>
+        </is>
+      </c>
+      <c r="E58" s="11" t="inlineStr">
+        <is>
+          <t>5.88</t>
+        </is>
+      </c>
+      <c r="F58" s="11" t="inlineStr">
+        <is>
+          <t>10.00%</t>
+        </is>
+      </c>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B59" s="10" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C59" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D59" s="11" t="inlineStr">
+        <is>
+          <t>19,200</t>
+        </is>
+      </c>
+      <c r="E59" s="11" t="inlineStr">
+        <is>
+          <t>5.71</t>
+        </is>
+      </c>
+      <c r="F59" s="11" t="inlineStr">
+        <is>
+          <t>10.50%</t>
+        </is>
+      </c>
+      <c r="G59" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>20,400</t>
+        </is>
+      </c>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>5.56</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>11.00%</t>
+        </is>
+      </c>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B61" s="10" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C61" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D61" s="11" t="inlineStr">
+        <is>
+          <t>21,600</t>
+        </is>
+      </c>
+      <c r="E61" s="11" t="inlineStr">
+        <is>
+          <t>5.41</t>
+        </is>
+      </c>
+      <c r="F61" s="11" t="inlineStr">
+        <is>
+          <t>11.50%</t>
+        </is>
+      </c>
+      <c r="G61" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>22,800</t>
+        </is>
+      </c>
+      <c r="E62" s="11" t="inlineStr">
+        <is>
+          <t>5.26</t>
+        </is>
+      </c>
+      <c r="F62" s="11" t="inlineStr">
+        <is>
+          <t>12.00%</t>
+        </is>
+      </c>
+      <c r="G62" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="10" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="B63" s="10" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>SOXL</t>
+        </is>
+      </c>
+      <c r="D63" s="11" t="inlineStr">
+        <is>
+          <t>24,000</t>
+        </is>
+      </c>
+      <c r="E63" s="11" t="inlineStr">
+        <is>
+          <t>5.13</t>
+        </is>
+      </c>
+      <c r="F63" s="11" t="inlineStr">
+        <is>
+          <t>12.50%</t>
+        </is>
+      </c>
+      <c r="G63" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Bybit BTCUSDT tier extraction using Chrome Channel and robust table locator
</commit_message>
<xml_diff>
--- a/data/all_exchanges_futures_margin.xlsx
+++ b/data/all_exchanges_futures_margin.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -2216,1221 +2216,1961 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>2,000,000</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>0.5%</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>2,600,000</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>0.56%</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>1,200</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>3,200,000</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>0.63%</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>3,020</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>3,800,000</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>0.67%</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>4,300</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>4,400,000</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>0.71%</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>5,820</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>5,000,000</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>0.77%</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>8,460</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>5,600,000</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>0.91%</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>15,460</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>8,500,000</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>20,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>10,000,000</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>1.3%</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>46,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>14,000,000</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>1.5%</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>66,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>20,000,000</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>1.6%</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>80,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>28,000,000</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>2%</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>160,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>38,000,000</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>2.5%</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>300,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>50,000,000</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>2.9%</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>452,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>55,000,000</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>502,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>60,000,000</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>3.5%</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>777,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>65,000,000</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>3.6%</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>837,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>70,000,000</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>3.8%</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>967,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>75,000,000</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>4%</t>
+        </is>
+      </c>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>1,107,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>80,000,000</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>4.5%</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>1,482,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
         <is>
           <t>MEXC</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B66" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C46" s="8" t="inlineStr">
+      <c r="C66" s="8" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D46" s="9" t="inlineStr">
+      <c r="D66" s="9" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E46" s="9" t="inlineStr">
+      <c r="E66" s="9" t="inlineStr">
         <is>
           <t>500x</t>
         </is>
       </c>
-      <c r="F46" s="9" t="inlineStr">
+      <c r="F66" s="9" t="inlineStr">
         <is>
           <t>0.1%</t>
         </is>
       </c>
-      <c r="G46" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="G66" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
         <is>
           <t>MEXC</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B67" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C47" s="8" t="inlineStr">
+      <c r="C67" s="8" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D47" s="9" t="inlineStr">
+      <c r="D67" s="9" t="inlineStr">
         <is>
           <t>31</t>
         </is>
       </c>
-      <c r="E47" s="9" t="inlineStr">
+      <c r="E67" s="9" t="inlineStr">
         <is>
           <t>200x</t>
         </is>
       </c>
-      <c r="F47" s="9" t="inlineStr">
+      <c r="F67" s="9" t="inlineStr">
         <is>
           <t>0.4%</t>
         </is>
       </c>
-      <c r="G47" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+      <c r="G67" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
         <is>
           <t>MEXC</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B68" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C48" s="8" t="inlineStr">
+      <c r="C68" s="8" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D48" s="9" t="inlineStr">
+      <c r="D68" s="9" t="inlineStr">
         <is>
           <t>48</t>
         </is>
       </c>
-      <c r="E48" s="9" t="inlineStr">
+      <c r="E68" s="9" t="inlineStr">
         <is>
           <t>100x</t>
         </is>
       </c>
-      <c r="F48" s="9" t="inlineStr">
+      <c r="F68" s="9" t="inlineStr">
         <is>
           <t>0.5%</t>
         </is>
       </c>
-      <c r="G48" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+      <c r="G68" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
         <is>
           <t>MEXC</t>
         </is>
       </c>
-      <c r="B49" s="8" t="inlineStr">
+      <c r="B69" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C49" s="8" t="inlineStr">
+      <c r="C69" s="8" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D49" s="9" t="inlineStr">
+      <c r="D69" s="9" t="inlineStr">
         <is>
           <t>280</t>
         </is>
       </c>
-      <c r="E49" s="9" t="inlineStr">
+      <c r="E69" s="9" t="inlineStr">
         <is>
           <t>50x</t>
         </is>
       </c>
-      <c r="F49" s="9" t="inlineStr">
+      <c r="F69" s="9" t="inlineStr">
         <is>
           <t>1%</t>
         </is>
       </c>
-      <c r="G49" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="G69" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
         <is>
           <t>MEXC</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B70" s="8" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C50" s="8" t="inlineStr">
+      <c r="C70" s="8" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D50" s="9" t="inlineStr">
+      <c r="D70" s="9" t="inlineStr">
         <is>
           <t>1,750</t>
         </is>
       </c>
-      <c r="E50" s="9" t="inlineStr">
+      <c r="E70" s="9" t="inlineStr">
         <is>
           <t>20x</t>
         </is>
       </c>
-      <c r="F50" s="9" t="inlineStr">
+      <c r="F70" s="9" t="inlineStr">
         <is>
           <t>2%</t>
         </is>
       </c>
-      <c r="G50" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="8" t="inlineStr">
+      <c r="G70" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
         <is>
           <t>MEXC</t>
         </is>
       </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="B71" s="8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C51" s="8" t="inlineStr">
+      <c r="C71" s="8" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D51" s="9" t="inlineStr">
+      <c r="D71" s="9" t="inlineStr">
         <is>
           <t>1,900</t>
         </is>
       </c>
-      <c r="E51" s="9" t="inlineStr">
+      <c r="E71" s="9" t="inlineStr">
         <is>
           <t>10x</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
+      <c r="F71" s="9" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="G51" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="10" t="inlineStr">
+      <c r="G71" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B52" s="10" t="inlineStr">
+      <c r="B72" s="10" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C52" s="10" t="inlineStr">
+      <c r="C72" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D52" s="11" t="inlineStr">
+      <c r="D72" s="11" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="E52" s="11" t="inlineStr">
+      <c r="E72" s="11" t="inlineStr">
         <is>
           <t>100.00</t>
         </is>
       </c>
-      <c r="F52" s="11" t="inlineStr">
+      <c r="F72" s="11" t="inlineStr">
         <is>
           <t>0.40%</t>
         </is>
       </c>
-      <c r="G52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="10" t="inlineStr">
+      <c r="G72" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B53" s="10" t="inlineStr">
+      <c r="B73" s="10" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="C53" s="10" t="inlineStr">
+      <c r="C73" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D53" s="11" t="inlineStr">
+      <c r="D73" s="11" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="E53" s="11" t="inlineStr">
+      <c r="E73" s="11" t="inlineStr">
         <is>
           <t>66.66</t>
         </is>
       </c>
-      <c r="F53" s="11" t="inlineStr">
+      <c r="F73" s="11" t="inlineStr">
         <is>
           <t>0.50%</t>
         </is>
       </c>
-      <c r="G53" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="10" t="inlineStr">
+      <c r="G73" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B54" s="10" t="inlineStr">
+      <c r="B74" s="10" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="C54" s="10" t="inlineStr">
+      <c r="C74" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D54" s="11" t="inlineStr">
+      <c r="D74" s="11" t="inlineStr">
         <is>
           <t>200</t>
         </is>
       </c>
-      <c r="E54" s="11" t="inlineStr">
+      <c r="E74" s="11" t="inlineStr">
         <is>
           <t>50.00</t>
         </is>
       </c>
-      <c r="F54" s="11" t="inlineStr">
+      <c r="F74" s="11" t="inlineStr">
         <is>
           <t>0.75%</t>
         </is>
       </c>
-      <c r="G54" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="10" t="inlineStr">
+      <c r="G74" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B55" s="10" t="inlineStr">
+      <c r="B75" s="10" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="C55" s="10" t="inlineStr">
+      <c r="C75" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D55" s="11" t="inlineStr">
+      <c r="D75" s="11" t="inlineStr">
         <is>
           <t>400</t>
         </is>
       </c>
-      <c r="E55" s="11" t="inlineStr">
+      <c r="E75" s="11" t="inlineStr">
         <is>
           <t>40.00</t>
         </is>
       </c>
-      <c r="F55" s="11" t="inlineStr">
+      <c r="F75" s="11" t="inlineStr">
         <is>
           <t>1.25%</t>
         </is>
       </c>
-      <c r="G55" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="10" t="inlineStr">
+      <c r="G75" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B56" s="10" t="inlineStr">
+      <c r="B76" s="10" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="C56" s="10" t="inlineStr">
+      <c r="C76" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D56" s="11" t="inlineStr">
+      <c r="D76" s="11" t="inlineStr">
         <is>
           <t>600</t>
         </is>
       </c>
-      <c r="E56" s="11" t="inlineStr">
+      <c r="E76" s="11" t="inlineStr">
         <is>
           <t>33.33</t>
         </is>
       </c>
-      <c r="F56" s="11" t="inlineStr">
+      <c r="F76" s="11" t="inlineStr">
         <is>
           <t>1.75%</t>
         </is>
       </c>
-      <c r="G56" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="10" t="inlineStr">
+      <c r="G76" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B57" s="10" t="inlineStr">
+      <c r="B77" s="10" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C57" s="10" t="inlineStr">
+      <c r="C77" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D57" s="11" t="inlineStr">
+      <c r="D77" s="11" t="inlineStr">
         <is>
           <t>800</t>
         </is>
       </c>
-      <c r="E57" s="11" t="inlineStr">
+      <c r="E77" s="11" t="inlineStr">
         <is>
           <t>28.57</t>
         </is>
       </c>
-      <c r="F57" s="11" t="inlineStr">
+      <c r="F77" s="11" t="inlineStr">
         <is>
           <t>2.25%</t>
         </is>
       </c>
-      <c r="G57" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="10" t="inlineStr">
+      <c r="G77" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B58" s="10" t="inlineStr">
+      <c r="B78" s="10" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="C58" s="10" t="inlineStr">
+      <c r="C78" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D58" s="11" t="inlineStr">
+      <c r="D78" s="11" t="inlineStr">
         <is>
           <t>1,000</t>
         </is>
       </c>
-      <c r="E58" s="11" t="inlineStr">
+      <c r="E78" s="11" t="inlineStr">
         <is>
           <t>25.00</t>
         </is>
       </c>
-      <c r="F58" s="11" t="inlineStr">
+      <c r="F78" s="11" t="inlineStr">
         <is>
           <t>2.75%</t>
         </is>
       </c>
-      <c r="G58" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="10" t="inlineStr">
+      <c r="G78" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B59" s="10" t="inlineStr">
+      <c r="B79" s="10" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C59" s="10" t="inlineStr">
+      <c r="C79" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D59" s="11" t="inlineStr">
+      <c r="D79" s="11" t="inlineStr">
         <is>
           <t>1,200</t>
         </is>
       </c>
-      <c r="E59" s="11" t="inlineStr">
+      <c r="E79" s="11" t="inlineStr">
         <is>
           <t>22.22</t>
         </is>
       </c>
-      <c r="F59" s="11" t="inlineStr">
+      <c r="F79" s="11" t="inlineStr">
         <is>
           <t>3.25%</t>
         </is>
       </c>
-      <c r="G59" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="10" t="inlineStr">
+      <c r="G79" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B60" s="10" t="inlineStr">
+      <c r="B80" s="10" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="C60" s="10" t="inlineStr">
+      <c r="C80" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D60" s="11" t="inlineStr">
+      <c r="D80" s="11" t="inlineStr">
         <is>
           <t>1,400</t>
         </is>
       </c>
-      <c r="E60" s="11" t="inlineStr">
+      <c r="E80" s="11" t="inlineStr">
         <is>
           <t>20.00</t>
         </is>
       </c>
-      <c r="F60" s="11" t="inlineStr">
+      <c r="F80" s="11" t="inlineStr">
         <is>
           <t>3.75%</t>
         </is>
       </c>
-      <c r="G60" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="10" t="inlineStr">
+      <c r="G80" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B61" s="10" t="inlineStr">
+      <c r="B81" s="10" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C61" s="10" t="inlineStr">
+      <c r="C81" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D61" s="11" t="inlineStr">
+      <c r="D81" s="11" t="inlineStr">
         <is>
           <t>1,600</t>
         </is>
       </c>
-      <c r="E61" s="11" t="inlineStr">
+      <c r="E81" s="11" t="inlineStr">
         <is>
           <t>18.18</t>
         </is>
       </c>
-      <c r="F61" s="11" t="inlineStr">
+      <c r="F81" s="11" t="inlineStr">
         <is>
           <t>4.25%</t>
         </is>
       </c>
-      <c r="G61" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="10" t="inlineStr">
+      <c r="G81" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B62" s="10" t="inlineStr">
+      <c r="B82" s="10" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="C62" s="10" t="inlineStr">
+      <c r="C82" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D62" s="11" t="inlineStr">
+      <c r="D82" s="11" t="inlineStr">
         <is>
           <t>1,800</t>
         </is>
       </c>
-      <c r="E62" s="11" t="inlineStr">
+      <c r="E82" s="11" t="inlineStr">
         <is>
           <t>16.66</t>
         </is>
       </c>
-      <c r="F62" s="11" t="inlineStr">
+      <c r="F82" s="11" t="inlineStr">
         <is>
           <t>4.75%</t>
         </is>
       </c>
-      <c r="G62" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="10" t="inlineStr">
+      <c r="G82" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B63" s="10" t="inlineStr">
+      <c r="B83" s="10" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="C63" s="10" t="inlineStr">
+      <c r="C83" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D63" s="11" t="inlineStr">
+      <c r="D83" s="11" t="inlineStr">
         <is>
           <t>2,000</t>
         </is>
       </c>
-      <c r="E63" s="11" t="inlineStr">
+      <c r="E83" s="11" t="inlineStr">
         <is>
           <t>15.38</t>
         </is>
       </c>
-      <c r="F63" s="11" t="inlineStr">
+      <c r="F83" s="11" t="inlineStr">
         <is>
           <t>5.25%</t>
         </is>
       </c>
-      <c r="G63" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="10" t="inlineStr">
+      <c r="G83" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B64" s="10" t="inlineStr">
+      <c r="B84" s="10" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="C64" s="10" t="inlineStr">
+      <c r="C84" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D64" s="11" t="inlineStr">
+      <c r="D84" s="11" t="inlineStr">
         <is>
           <t>2,200</t>
         </is>
       </c>
-      <c r="E64" s="11" t="inlineStr">
+      <c r="E84" s="11" t="inlineStr">
         <is>
           <t>14.28</t>
         </is>
       </c>
-      <c r="F64" s="11" t="inlineStr">
+      <c r="F84" s="11" t="inlineStr">
         <is>
           <t>5.75%</t>
         </is>
       </c>
-      <c r="G64" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="10" t="inlineStr">
+      <c r="G84" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B65" s="10" t="inlineStr">
+      <c r="B85" s="10" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="C65" s="10" t="inlineStr">
+      <c r="C85" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D65" s="11" t="inlineStr">
+      <c r="D85" s="11" t="inlineStr">
         <is>
           <t>2,400</t>
         </is>
       </c>
-      <c r="E65" s="11" t="inlineStr">
+      <c r="E85" s="11" t="inlineStr">
         <is>
           <t>13.33</t>
         </is>
       </c>
-      <c r="F65" s="11" t="inlineStr">
+      <c r="F85" s="11" t="inlineStr">
         <is>
           <t>6.25%</t>
         </is>
       </c>
-      <c r="G65" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="10" t="inlineStr">
+      <c r="G85" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B66" s="10" t="inlineStr">
+      <c r="B86" s="10" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="C66" s="10" t="inlineStr">
+      <c r="C86" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D66" s="11" t="inlineStr">
+      <c r="D86" s="11" t="inlineStr">
         <is>
           <t>2,600</t>
         </is>
       </c>
-      <c r="E66" s="11" t="inlineStr">
+      <c r="E86" s="11" t="inlineStr">
         <is>
           <t>12.50</t>
         </is>
       </c>
-      <c r="F66" s="11" t="inlineStr">
+      <c r="F86" s="11" t="inlineStr">
         <is>
           <t>6.75%</t>
         </is>
       </c>
-      <c r="G66" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="10" t="inlineStr">
+      <c r="G86" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B67" s="10" t="inlineStr">
+      <c r="B87" s="10" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="C67" s="10" t="inlineStr">
+      <c r="C87" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D67" s="11" t="inlineStr">
+      <c r="D87" s="11" t="inlineStr">
         <is>
           <t>2,800</t>
         </is>
       </c>
-      <c r="E67" s="11" t="inlineStr">
+      <c r="E87" s="11" t="inlineStr">
         <is>
           <t>11.76</t>
         </is>
       </c>
-      <c r="F67" s="11" t="inlineStr">
+      <c r="F87" s="11" t="inlineStr">
         <is>
           <t>7.25%</t>
         </is>
       </c>
-      <c r="G67" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="10" t="inlineStr">
+      <c r="G87" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B68" s="10" t="inlineStr">
+      <c r="B88" s="10" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="C68" s="10" t="inlineStr">
+      <c r="C88" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D68" s="11" t="inlineStr">
+      <c r="D88" s="11" t="inlineStr">
         <is>
           <t>3,000</t>
         </is>
       </c>
-      <c r="E68" s="11" t="inlineStr">
+      <c r="E88" s="11" t="inlineStr">
         <is>
           <t>11.11</t>
         </is>
       </c>
-      <c r="F68" s="11" t="inlineStr">
+      <c r="F88" s="11" t="inlineStr">
         <is>
           <t>7.75%</t>
         </is>
       </c>
-      <c r="G68" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="10" t="inlineStr">
+      <c r="G88" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B69" s="10" t="inlineStr">
+      <c r="B89" s="10" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="C69" s="10" t="inlineStr">
+      <c r="C89" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D69" s="11" t="inlineStr">
+      <c r="D89" s="11" t="inlineStr">
         <is>
           <t>3,200</t>
         </is>
       </c>
-      <c r="E69" s="11" t="inlineStr">
+      <c r="E89" s="11" t="inlineStr">
         <is>
           <t>10.52</t>
         </is>
       </c>
-      <c r="F69" s="11" t="inlineStr">
+      <c r="F89" s="11" t="inlineStr">
         <is>
           <t>8.25%</t>
         </is>
       </c>
-      <c r="G69" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="10" t="inlineStr">
+      <c r="G89" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B70" s="10" t="inlineStr">
+      <c r="B90" s="10" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="C70" s="10" t="inlineStr">
+      <c r="C90" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D70" s="11" t="inlineStr">
+      <c r="D90" s="11" t="inlineStr">
         <is>
           <t>3,400</t>
         </is>
       </c>
-      <c r="E70" s="11" t="inlineStr">
+      <c r="E90" s="11" t="inlineStr">
         <is>
           <t>10.00</t>
         </is>
       </c>
-      <c r="F70" s="11" t="inlineStr">
+      <c r="F90" s="11" t="inlineStr">
         <is>
           <t>8.75%</t>
         </is>
       </c>
-      <c r="G70" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="10" t="inlineStr">
+      <c r="G90" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="10" t="inlineStr">
         <is>
           <t>OKX</t>
         </is>
       </c>
-      <c r="B71" s="10" t="inlineStr">
+      <c r="B91" s="10" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="C71" s="10" t="inlineStr">
+      <c r="C91" s="10" t="inlineStr">
         <is>
           <t>BTC</t>
         </is>
       </c>
-      <c r="D71" s="11" t="inlineStr">
+      <c r="D91" s="11" t="inlineStr">
         <is>
           <t>3,600</t>
         </is>
       </c>
-      <c r="E71" s="11" t="inlineStr">
+      <c r="E91" s="11" t="inlineStr">
         <is>
           <t>9.52</t>
         </is>
       </c>
-      <c r="F71" s="11" t="inlineStr">
+      <c r="F91" s="11" t="inlineStr">
         <is>
           <t>9.25%</t>
         </is>
       </c>
-      <c r="G71" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="14" t="inlineStr">
+      <c r="G91" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="14" t="inlineStr">
         <is>
           <t>Pionex (派網)</t>
         </is>
       </c>
-      <c r="B72" s="14" t="inlineStr">
+      <c r="B92" s="14" t="inlineStr">
         <is>
           <t>檔位 1</t>
         </is>
       </c>
-      <c r="C72" s="14" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="D72" s="15" t="inlineStr">
+      <c r="C92" s="14" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D92" s="15" t="inlineStr">
         <is>
           <t>2,000,000</t>
         </is>
       </c>
-      <c r="E72" s="15" t="inlineStr">
+      <c r="E92" s="15" t="inlineStr">
         <is>
           <t>100x</t>
         </is>
       </c>
-      <c r="F72" s="15" t="inlineStr">
+      <c r="F92" s="15" t="inlineStr">
         <is>
           <t>0.50%</t>
         </is>
       </c>
-      <c r="G72" s="15" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="14" t="inlineStr">
+      <c r="G92" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="14" t="inlineStr">
         <is>
           <t>Pionex (派網)</t>
         </is>
       </c>
-      <c r="B73" s="14" t="inlineStr">
+      <c r="B93" s="14" t="inlineStr">
         <is>
           <t>檔位 2</t>
         </is>
       </c>
-      <c r="C73" s="14" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="D73" s="15" t="inlineStr">
+      <c r="C93" s="14" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D93" s="15" t="inlineStr">
         <is>
           <t>12,000,000</t>
         </is>
       </c>
-      <c r="E73" s="15" t="inlineStr">
+      <c r="E93" s="15" t="inlineStr">
         <is>
           <t>50x</t>
         </is>
       </c>
-      <c r="F73" s="15" t="inlineStr">
+      <c r="F93" s="15" t="inlineStr">
         <is>
           <t>1.00%</t>
         </is>
       </c>
-      <c r="G73" s="15" t="inlineStr">
+      <c r="G93" s="15" t="inlineStr">
         <is>
           <t>10,000</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="14" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="14" t="inlineStr">
         <is>
           <t>Pionex (派網)</t>
         </is>
       </c>
-      <c r="B74" s="14" t="inlineStr">
+      <c r="B94" s="14" t="inlineStr">
         <is>
           <t>檔位 3</t>
         </is>
       </c>
-      <c r="C74" s="14" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="D74" s="15" t="inlineStr">
+      <c r="C94" s="14" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D94" s="15" t="inlineStr">
         <is>
           <t>100,000,000</t>
         </is>
       </c>
-      <c r="E74" s="15" t="inlineStr">
+      <c r="E94" s="15" t="inlineStr">
         <is>
           <t>20x</t>
         </is>
       </c>
-      <c r="F74" s="15" t="inlineStr">
+      <c r="F94" s="15" t="inlineStr">
         <is>
           <t>2.50%</t>
         </is>
       </c>
-      <c r="G74" s="15" t="inlineStr">
+      <c r="G94" s="15" t="inlineStr">
         <is>
           <t>190,000</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="14" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="14" t="inlineStr">
         <is>
           <t>Pionex (派網)</t>
         </is>
       </c>
-      <c r="B75" s="14" t="inlineStr">
+      <c r="B95" s="14" t="inlineStr">
         <is>
           <t>檔位 4</t>
         </is>
       </c>
-      <c r="C75" s="14" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="D75" s="15" t="inlineStr">
+      <c r="C95" s="14" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D95" s="15" t="inlineStr">
         <is>
           <t>200,000,000</t>
         </is>
       </c>
-      <c r="E75" s="15" t="inlineStr">
+      <c r="E95" s="15" t="inlineStr">
         <is>
           <t>10x</t>
         </is>
       </c>
-      <c r="F75" s="15" t="inlineStr">
+      <c r="F95" s="15" t="inlineStr">
         <is>
           <t>5.00%</t>
         </is>
       </c>
-      <c r="G75" s="15" t="inlineStr">
+      <c r="G95" s="15" t="inlineStr">
         <is>
           <t>2,690,000</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="14" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="14" t="inlineStr">
         <is>
           <t>Pionex (派網)</t>
         </is>
       </c>
-      <c r="B76" s="14" t="inlineStr">
+      <c r="B96" s="14" t="inlineStr">
         <is>
           <t>檔位 5</t>
         </is>
       </c>
-      <c r="C76" s="14" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="D76" s="15" t="inlineStr">
+      <c r="C96" s="14" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D96" s="15" t="inlineStr">
         <is>
           <t>500,000,000</t>
         </is>
       </c>
-      <c r="E76" s="15" t="inlineStr">
+      <c r="E96" s="15" t="inlineStr">
         <is>
           <t>5x</t>
         </is>
       </c>
-      <c r="F76" s="15" t="inlineStr">
+      <c r="F96" s="15" t="inlineStr">
         <is>
           <t>10.00%</t>
         </is>
       </c>
-      <c r="G76" s="15" t="inlineStr">
+      <c r="G96" s="15" t="inlineStr">
         <is>
           <t>12,690,000</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="14" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="14" t="inlineStr">
         <is>
           <t>Pionex (派網)</t>
         </is>
       </c>
-      <c r="B77" s="14" t="inlineStr">
+      <c r="B97" s="14" t="inlineStr">
         <is>
           <t>檔位 6</t>
         </is>
       </c>
-      <c r="C77" s="14" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="D77" s="15" t="inlineStr">
+      <c r="C97" s="14" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D97" s="15" t="inlineStr">
         <is>
           <t>600,000,000</t>
         </is>
       </c>
-      <c r="E77" s="15" t="inlineStr">
+      <c r="E97" s="15" t="inlineStr">
         <is>
           <t>2x</t>
         </is>
       </c>
-      <c r="F77" s="15" t="inlineStr">
+      <c r="F97" s="15" t="inlineStr">
         <is>
           <t>25.00%</t>
         </is>
       </c>
-      <c r="G77" s="15" t="inlineStr">
+      <c r="G97" s="15" t="inlineStr">
         <is>
           <t>87,690,000</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="14" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="14" t="inlineStr">
         <is>
           <t>Pionex (派網)</t>
         </is>
       </c>
-      <c r="B78" s="14" t="inlineStr">
+      <c r="B98" s="14" t="inlineStr">
         <is>
           <t>檔位 7</t>
         </is>
       </c>
-      <c r="C78" s="14" t="inlineStr">
-        <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="D78" s="15" t="inlineStr">
+      <c r="C98" s="14" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="D98" s="15" t="inlineStr">
         <is>
           <t>800,000,000</t>
         </is>
       </c>
-      <c r="E78" s="15" t="inlineStr">
+      <c r="E98" s="15" t="inlineStr">
         <is>
           <t>1x</t>
         </is>
       </c>
-      <c r="F78" s="15" t="inlineStr">
+      <c r="F98" s="15" t="inlineStr">
         <is>
           <t>50.00%</t>
         </is>
       </c>
-      <c r="G78" s="15" t="inlineStr">
+      <c r="G98" s="15" t="inlineStr">
         <is>
           <t>237,690,000</t>
         </is>

</xml_diff>